<commit_message>
Add fire group roster and duty sheet to June 2026 table
New "Склад МВГ" sheet lists each group's members (position, rank,
full name, callsign) with a 30-day grid for marking who was on a
mission each day. Per-person days, daily headcount per group and
person-days are calculated by formulas, and the summary sheet now
shows headcount and person-days per group. The daily hits sheet is
unchanged, so data already entered can be copied over as is.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WTuZ4H7b2ZscwX4NGxpWXu
</commit_message>
<xml_diff>
--- a/reports/mobile-fire-groups-2026-06.xlsx
+++ b/reports/mobile-fire-groups-2026-06.xlsx
@@ -9,9 +9,11 @@
   </bookViews>
   <sheets>
     <sheet name="Щоденний облік" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Підсумок" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Склад МВГ" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Підсумок" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">'Склад МВГ'!$4:$6</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Щоденний облік'!$4:$5</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -24,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="62">
   <si>
     <t xml:space="preserve">Облік виконання завдань мобільними вогневими групами «СТАЯ», «РОМБ», «ДАЧА» за червень 2026 року</t>
   </si>
@@ -104,6 +106,78 @@
     <t xml:space="preserve">Склав: ____________________________   ____________   «____» ____________ 2026 р.</t>
   </si>
   <si>
+    <t xml:space="preserve">Склад мобільних вогневих груп «СТАЯ», «РОМБ», «ДАЧА» та участь у виконанні завдань за червень 2026 року</t>
+  </si>
+  <si>
+    <t xml:space="preserve">У стовпцях днів поставте «+», якщо військовослужбовець того дня виконував завдання у складі МВГ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Посада в групі</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Військове звання</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Прізвище, ім'я, по батькові</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Позивний</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Дні виконання завдань — червень 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Всього діб на завданні</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Разом на завданні у МВГ «СТАЯ», осіб (за добу) / людино-діб</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Разом на завданні у МВГ «РОМБ», осіб (за добу) / людино-діб</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Разом на завданні у МВГ «ДАЧА», осіб (за добу) / людино-діб</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ВСЬОГО на завданні по МВГ, осіб (за добу) / людино-діб</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Жовті клітинки — посада, звання, П.І.Б., позивний кожного члена групи (посаду та звання можна вибрати зі списку або вписати вручну).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. У стовпцях днів ставте «+» у ті дні, коли військовослужбовець виконував завдання у складі цієї МВГ.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Кількість особового складу, «Всього діб», рядки «Разом на завданні» та «ВСЬОГО» рахуються автоматично — не редагувати.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Потрібно більше 10 осіб у групі — вставте рядок усередині блоку групи (між першим і останнім рядком), формули розширяться самі.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Якщо військовослужбовець протягом місяця працював у різних МВГ — впишіть його в кожну групу з відповідними днями.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Приклад заповнення рядка (умовні дані, у підрахунках не враховується):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Старший групи</t>
+  </si>
+  <si>
+    <t xml:space="preserve">старший солдат</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Петренко Петро Петрович</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сокіл</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">з 08.06 — відрядження</t>
+  </si>
+  <si>
     <t xml:space="preserve">Підсумок виконання завдань МВГ «СТАЯ», «РОМБ», «ДАЧА» за червень 2026 року</t>
   </si>
   <si>
@@ -117,6 +191,12 @@
   </si>
   <si>
     <t xml:space="preserve">Найрезультативніша доба</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Особовий склад, осіб</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Людино-діб на завданні</t>
   </si>
   <si>
     <t xml:space="preserve">Розподіл уражень за декадами (разом по всіх типах цілей)</t>
@@ -134,22 +214,23 @@
 21–30.06</t>
   </si>
   <si>
-    <t xml:space="preserve">Усі значення на цьому аркуші розраховуються автоматично з аркуша «Щоденний облік».</t>
+    <t xml:space="preserve">Усі значення на цьому аркуші розраховуються автоматично з аркушів «Щоденний облік» та «Склад МВГ».</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="dd\.mm\.yyyy"/>
     <numFmt numFmtId="166" formatCode="General"/>
     <numFmt numFmtId="167" formatCode="0"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
-    <numFmt numFmtId="169" formatCode="0.0%"/>
+    <numFmt numFmtId="169" formatCode="0;\-0;;@"/>
+    <numFmt numFmtId="170" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -238,6 +319,14 @@
       <i val="true"/>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -378,7 +467,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="55">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -495,7 +584,55 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -511,7 +648,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -531,7 +668,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -543,11 +680,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2798,7 +2935,2526 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:AK55"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="6" style="0" width="3.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="0" width="24"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
+      <c r="AE1" s="1"/>
+      <c r="AF1" s="1"/>
+      <c r="AG1" s="1"/>
+      <c r="AH1" s="1"/>
+      <c r="AI1" s="1"/>
+      <c r="AJ1" s="1"/>
+      <c r="AK1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2"/>
+      <c r="V2" s="2"/>
+      <c r="W2" s="2"/>
+      <c r="X2" s="2"/>
+      <c r="Y2" s="2"/>
+      <c r="Z2" s="2"/>
+      <c r="AA2" s="2"/>
+      <c r="AB2" s="2"/>
+      <c r="AC2" s="2"/>
+      <c r="AD2" s="2"/>
+      <c r="AE2" s="2"/>
+      <c r="AF2" s="2"/>
+      <c r="AG2" s="2"/>
+      <c r="AH2" s="2"/>
+      <c r="AI2" s="2"/>
+      <c r="AJ2" s="2"/>
+      <c r="AK2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="3"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+      <c r="Y4" s="3"/>
+      <c r="Z4" s="3"/>
+      <c r="AA4" s="3"/>
+      <c r="AB4" s="3"/>
+      <c r="AC4" s="3"/>
+      <c r="AD4" s="3"/>
+      <c r="AE4" s="3"/>
+      <c r="AF4" s="3"/>
+      <c r="AG4" s="3"/>
+      <c r="AH4" s="3"/>
+      <c r="AI4" s="3"/>
+      <c r="AJ4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="AK4" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="R5" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="S5" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="T5" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="U5" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="V5" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="W5" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="X5" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="Y5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="Z5" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="AA5" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="AB5" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="AC5" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="AD5" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="AE5" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="AF5" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="AG5" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="AH5" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="AI5" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="AJ5" s="3"/>
+      <c r="AK5" s="3"/>
+    </row>
+    <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,F$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Пн</v>
+      </c>
+      <c r="G6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,G$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Вт</v>
+      </c>
+      <c r="H6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,H$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Ср</v>
+      </c>
+      <c r="I6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,I$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Чт</v>
+      </c>
+      <c r="J6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,J$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Пт</v>
+      </c>
+      <c r="K6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,K$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Сб</v>
+      </c>
+      <c r="L6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,L$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Нд</v>
+      </c>
+      <c r="M6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,M$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Пн</v>
+      </c>
+      <c r="N6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,N$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Вт</v>
+      </c>
+      <c r="O6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,O$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Ср</v>
+      </c>
+      <c r="P6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,P$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Чт</v>
+      </c>
+      <c r="Q6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,Q$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Пт</v>
+      </c>
+      <c r="R6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,R$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Сб</v>
+      </c>
+      <c r="S6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,S$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Нд</v>
+      </c>
+      <c r="T6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,T$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Пн</v>
+      </c>
+      <c r="U6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,U$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Вт</v>
+      </c>
+      <c r="V6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,V$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Ср</v>
+      </c>
+      <c r="W6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,W$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Чт</v>
+      </c>
+      <c r="X6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,X$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Пт</v>
+      </c>
+      <c r="Y6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,Y$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Сб</v>
+      </c>
+      <c r="Z6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,Z$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Нд</v>
+      </c>
+      <c r="AA6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,AA$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Пн</v>
+      </c>
+      <c r="AB6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,AB$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Вт</v>
+      </c>
+      <c r="AC6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,AC$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Ср</v>
+      </c>
+      <c r="AD6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,AD$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Чт</v>
+      </c>
+      <c r="AE6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,AE$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Пт</v>
+      </c>
+      <c r="AF6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,AF$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Сб</v>
+      </c>
+      <c r="AG6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,AG$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Нд</v>
+      </c>
+      <c r="AH6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,AH$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Пн</v>
+      </c>
+      <c r="AI6" s="29" t="str">
+        <f aca="false">CHOOSE(WEEKDAY(DATE(2026,6,AI$5),2),"Пн","Вт","Ср","Чт","Пт","Сб","Нд")</f>
+        <v>Вт</v>
+      </c>
+      <c r="AJ6" s="3"/>
+      <c r="AK6" s="3"/>
+    </row>
+    <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="30" t="str">
+        <f aca="false">"МВГ «СТАЯ» — особовий склад, осіб: "&amp;COUNTA(D8:D17)</f>
+        <v>МВГ «СТАЯ» — особовий склад, осіб: 0</v>
+      </c>
+      <c r="B7" s="30"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="30"/>
+      <c r="J7" s="30"/>
+      <c r="K7" s="30"/>
+      <c r="L7" s="30"/>
+      <c r="M7" s="30"/>
+      <c r="N7" s="30"/>
+      <c r="O7" s="30"/>
+      <c r="P7" s="30"/>
+      <c r="Q7" s="30"/>
+      <c r="R7" s="30"/>
+      <c r="S7" s="30"/>
+      <c r="T7" s="30"/>
+      <c r="U7" s="30"/>
+      <c r="V7" s="30"/>
+      <c r="W7" s="30"/>
+      <c r="X7" s="30"/>
+      <c r="Y7" s="30"/>
+      <c r="Z7" s="30"/>
+      <c r="AA7" s="30"/>
+      <c r="AB7" s="30"/>
+      <c r="AC7" s="30"/>
+      <c r="AD7" s="30"/>
+      <c r="AE7" s="30"/>
+      <c r="AF7" s="30"/>
+      <c r="AG7" s="30"/>
+      <c r="AH7" s="30"/>
+      <c r="AI7" s="30"/>
+      <c r="AJ7" s="30"/>
+      <c r="AK7" s="30"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="31"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="31"/>
+      <c r="E8" s="31"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="10"/>
+      <c r="P8" s="10"/>
+      <c r="Q8" s="10"/>
+      <c r="R8" s="10"/>
+      <c r="S8" s="10"/>
+      <c r="T8" s="10"/>
+      <c r="U8" s="10"/>
+      <c r="V8" s="10"/>
+      <c r="W8" s="10"/>
+      <c r="X8" s="10"/>
+      <c r="Y8" s="10"/>
+      <c r="Z8" s="10"/>
+      <c r="AA8" s="10"/>
+      <c r="AB8" s="10"/>
+      <c r="AC8" s="10"/>
+      <c r="AD8" s="10"/>
+      <c r="AE8" s="10"/>
+      <c r="AF8" s="10"/>
+      <c r="AG8" s="10"/>
+      <c r="AH8" s="10"/>
+      <c r="AI8" s="10"/>
+      <c r="AJ8" s="32" t="n">
+        <f aca="false">COUNTA(F8:AI8)</f>
+        <v>0</v>
+      </c>
+      <c r="AK8" s="33"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="31"/>
+      <c r="C9" s="31"/>
+      <c r="D9" s="31"/>
+      <c r="E9" s="31"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
+      <c r="O9" s="10"/>
+      <c r="P9" s="10"/>
+      <c r="Q9" s="10"/>
+      <c r="R9" s="10"/>
+      <c r="S9" s="10"/>
+      <c r="T9" s="10"/>
+      <c r="U9" s="10"/>
+      <c r="V9" s="10"/>
+      <c r="W9" s="10"/>
+      <c r="X9" s="10"/>
+      <c r="Y9" s="10"/>
+      <c r="Z9" s="10"/>
+      <c r="AA9" s="10"/>
+      <c r="AB9" s="10"/>
+      <c r="AC9" s="10"/>
+      <c r="AD9" s="10"/>
+      <c r="AE9" s="10"/>
+      <c r="AF9" s="10"/>
+      <c r="AG9" s="10"/>
+      <c r="AH9" s="10"/>
+      <c r="AI9" s="10"/>
+      <c r="AJ9" s="32" t="n">
+        <f aca="false">COUNTA(F9:AI9)</f>
+        <v>0</v>
+      </c>
+      <c r="AK9" s="33"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="31"/>
+      <c r="C10" s="31"/>
+      <c r="D10" s="31"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
+      <c r="O10" s="10"/>
+      <c r="P10" s="10"/>
+      <c r="Q10" s="10"/>
+      <c r="R10" s="10"/>
+      <c r="S10" s="10"/>
+      <c r="T10" s="10"/>
+      <c r="U10" s="10"/>
+      <c r="V10" s="10"/>
+      <c r="W10" s="10"/>
+      <c r="X10" s="10"/>
+      <c r="Y10" s="10"/>
+      <c r="Z10" s="10"/>
+      <c r="AA10" s="10"/>
+      <c r="AB10" s="10"/>
+      <c r="AC10" s="10"/>
+      <c r="AD10" s="10"/>
+      <c r="AE10" s="10"/>
+      <c r="AF10" s="10"/>
+      <c r="AG10" s="10"/>
+      <c r="AH10" s="10"/>
+      <c r="AI10" s="10"/>
+      <c r="AJ10" s="32" t="n">
+        <f aca="false">COUNTA(F10:AI10)</f>
+        <v>0</v>
+      </c>
+      <c r="AK10" s="33"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" s="31"/>
+      <c r="C11" s="31"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="31"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="10"/>
+      <c r="O11" s="10"/>
+      <c r="P11" s="10"/>
+      <c r="Q11" s="10"/>
+      <c r="R11" s="10"/>
+      <c r="S11" s="10"/>
+      <c r="T11" s="10"/>
+      <c r="U11" s="10"/>
+      <c r="V11" s="10"/>
+      <c r="W11" s="10"/>
+      <c r="X11" s="10"/>
+      <c r="Y11" s="10"/>
+      <c r="Z11" s="10"/>
+      <c r="AA11" s="10"/>
+      <c r="AB11" s="10"/>
+      <c r="AC11" s="10"/>
+      <c r="AD11" s="10"/>
+      <c r="AE11" s="10"/>
+      <c r="AF11" s="10"/>
+      <c r="AG11" s="10"/>
+      <c r="AH11" s="10"/>
+      <c r="AI11" s="10"/>
+      <c r="AJ11" s="32" t="n">
+        <f aca="false">COUNTA(F11:AI11)</f>
+        <v>0</v>
+      </c>
+      <c r="AK11" s="33"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" s="31"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="10"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="10"/>
+      <c r="O12" s="10"/>
+      <c r="P12" s="10"/>
+      <c r="Q12" s="10"/>
+      <c r="R12" s="10"/>
+      <c r="S12" s="10"/>
+      <c r="T12" s="10"/>
+      <c r="U12" s="10"/>
+      <c r="V12" s="10"/>
+      <c r="W12" s="10"/>
+      <c r="X12" s="10"/>
+      <c r="Y12" s="10"/>
+      <c r="Z12" s="10"/>
+      <c r="AA12" s="10"/>
+      <c r="AB12" s="10"/>
+      <c r="AC12" s="10"/>
+      <c r="AD12" s="10"/>
+      <c r="AE12" s="10"/>
+      <c r="AF12" s="10"/>
+      <c r="AG12" s="10"/>
+      <c r="AH12" s="10"/>
+      <c r="AI12" s="10"/>
+      <c r="AJ12" s="32" t="n">
+        <f aca="false">COUNTA(F12:AI12)</f>
+        <v>0</v>
+      </c>
+      <c r="AK12" s="33"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" s="31"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10"/>
+      <c r="L13" s="10"/>
+      <c r="M13" s="10"/>
+      <c r="N13" s="10"/>
+      <c r="O13" s="10"/>
+      <c r="P13" s="10"/>
+      <c r="Q13" s="10"/>
+      <c r="R13" s="10"/>
+      <c r="S13" s="10"/>
+      <c r="T13" s="10"/>
+      <c r="U13" s="10"/>
+      <c r="V13" s="10"/>
+      <c r="W13" s="10"/>
+      <c r="X13" s="10"/>
+      <c r="Y13" s="10"/>
+      <c r="Z13" s="10"/>
+      <c r="AA13" s="10"/>
+      <c r="AB13" s="10"/>
+      <c r="AC13" s="10"/>
+      <c r="AD13" s="10"/>
+      <c r="AE13" s="10"/>
+      <c r="AF13" s="10"/>
+      <c r="AG13" s="10"/>
+      <c r="AH13" s="10"/>
+      <c r="AI13" s="10"/>
+      <c r="AJ13" s="32" t="n">
+        <f aca="false">COUNTA(F13:AI13)</f>
+        <v>0</v>
+      </c>
+      <c r="AK13" s="33"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B14" s="31"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="31"/>
+      <c r="E14" s="31"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="10"/>
+      <c r="O14" s="10"/>
+      <c r="P14" s="10"/>
+      <c r="Q14" s="10"/>
+      <c r="R14" s="10"/>
+      <c r="S14" s="10"/>
+      <c r="T14" s="10"/>
+      <c r="U14" s="10"/>
+      <c r="V14" s="10"/>
+      <c r="W14" s="10"/>
+      <c r="X14" s="10"/>
+      <c r="Y14" s="10"/>
+      <c r="Z14" s="10"/>
+      <c r="AA14" s="10"/>
+      <c r="AB14" s="10"/>
+      <c r="AC14" s="10"/>
+      <c r="AD14" s="10"/>
+      <c r="AE14" s="10"/>
+      <c r="AF14" s="10"/>
+      <c r="AG14" s="10"/>
+      <c r="AH14" s="10"/>
+      <c r="AI14" s="10"/>
+      <c r="AJ14" s="32" t="n">
+        <f aca="false">COUNTA(F14:AI14)</f>
+        <v>0</v>
+      </c>
+      <c r="AK14" s="33"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B15" s="31"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
+      <c r="O15" s="10"/>
+      <c r="P15" s="10"/>
+      <c r="Q15" s="10"/>
+      <c r="R15" s="10"/>
+      <c r="S15" s="10"/>
+      <c r="T15" s="10"/>
+      <c r="U15" s="10"/>
+      <c r="V15" s="10"/>
+      <c r="W15" s="10"/>
+      <c r="X15" s="10"/>
+      <c r="Y15" s="10"/>
+      <c r="Z15" s="10"/>
+      <c r="AA15" s="10"/>
+      <c r="AB15" s="10"/>
+      <c r="AC15" s="10"/>
+      <c r="AD15" s="10"/>
+      <c r="AE15" s="10"/>
+      <c r="AF15" s="10"/>
+      <c r="AG15" s="10"/>
+      <c r="AH15" s="10"/>
+      <c r="AI15" s="10"/>
+      <c r="AJ15" s="32" t="n">
+        <f aca="false">COUNTA(F15:AI15)</f>
+        <v>0</v>
+      </c>
+      <c r="AK15" s="33"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="B16" s="31"/>
+      <c r="C16" s="31"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="10"/>
+      <c r="L16" s="10"/>
+      <c r="M16" s="10"/>
+      <c r="N16" s="10"/>
+      <c r="O16" s="10"/>
+      <c r="P16" s="10"/>
+      <c r="Q16" s="10"/>
+      <c r="R16" s="10"/>
+      <c r="S16" s="10"/>
+      <c r="T16" s="10"/>
+      <c r="U16" s="10"/>
+      <c r="V16" s="10"/>
+      <c r="W16" s="10"/>
+      <c r="X16" s="10"/>
+      <c r="Y16" s="10"/>
+      <c r="Z16" s="10"/>
+      <c r="AA16" s="10"/>
+      <c r="AB16" s="10"/>
+      <c r="AC16" s="10"/>
+      <c r="AD16" s="10"/>
+      <c r="AE16" s="10"/>
+      <c r="AF16" s="10"/>
+      <c r="AG16" s="10"/>
+      <c r="AH16" s="10"/>
+      <c r="AI16" s="10"/>
+      <c r="AJ16" s="32" t="n">
+        <f aca="false">COUNTA(F16:AI16)</f>
+        <v>0</v>
+      </c>
+      <c r="AK16" s="33"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B17" s="31"/>
+      <c r="C17" s="31"/>
+      <c r="D17" s="31"/>
+      <c r="E17" s="31"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="10"/>
+      <c r="L17" s="10"/>
+      <c r="M17" s="10"/>
+      <c r="N17" s="10"/>
+      <c r="O17" s="10"/>
+      <c r="P17" s="10"/>
+      <c r="Q17" s="10"/>
+      <c r="R17" s="10"/>
+      <c r="S17" s="10"/>
+      <c r="T17" s="10"/>
+      <c r="U17" s="10"/>
+      <c r="V17" s="10"/>
+      <c r="W17" s="10"/>
+      <c r="X17" s="10"/>
+      <c r="Y17" s="10"/>
+      <c r="Z17" s="10"/>
+      <c r="AA17" s="10"/>
+      <c r="AB17" s="10"/>
+      <c r="AC17" s="10"/>
+      <c r="AD17" s="10"/>
+      <c r="AE17" s="10"/>
+      <c r="AF17" s="10"/>
+      <c r="AG17" s="10"/>
+      <c r="AH17" s="10"/>
+      <c r="AI17" s="10"/>
+      <c r="AJ17" s="32" t="n">
+        <f aca="false">COUNTA(F17:AI17)</f>
+        <v>0</v>
+      </c>
+      <c r="AK17" s="33"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="34" t="n">
+        <f aca="false">COUNTA(F8:F17)</f>
+        <v>0</v>
+      </c>
+      <c r="G18" s="34" t="n">
+        <f aca="false">COUNTA(G8:G17)</f>
+        <v>0</v>
+      </c>
+      <c r="H18" s="34" t="n">
+        <f aca="false">COUNTA(H8:H17)</f>
+        <v>0</v>
+      </c>
+      <c r="I18" s="34" t="n">
+        <f aca="false">COUNTA(I8:I17)</f>
+        <v>0</v>
+      </c>
+      <c r="J18" s="34" t="n">
+        <f aca="false">COUNTA(J8:J17)</f>
+        <v>0</v>
+      </c>
+      <c r="K18" s="34" t="n">
+        <f aca="false">COUNTA(K8:K17)</f>
+        <v>0</v>
+      </c>
+      <c r="L18" s="34" t="n">
+        <f aca="false">COUNTA(L8:L17)</f>
+        <v>0</v>
+      </c>
+      <c r="M18" s="34" t="n">
+        <f aca="false">COUNTA(M8:M17)</f>
+        <v>0</v>
+      </c>
+      <c r="N18" s="34" t="n">
+        <f aca="false">COUNTA(N8:N17)</f>
+        <v>0</v>
+      </c>
+      <c r="O18" s="34" t="n">
+        <f aca="false">COUNTA(O8:O17)</f>
+        <v>0</v>
+      </c>
+      <c r="P18" s="34" t="n">
+        <f aca="false">COUNTA(P8:P17)</f>
+        <v>0</v>
+      </c>
+      <c r="Q18" s="34" t="n">
+        <f aca="false">COUNTA(Q8:Q17)</f>
+        <v>0</v>
+      </c>
+      <c r="R18" s="34" t="n">
+        <f aca="false">COUNTA(R8:R17)</f>
+        <v>0</v>
+      </c>
+      <c r="S18" s="34" t="n">
+        <f aca="false">COUNTA(S8:S17)</f>
+        <v>0</v>
+      </c>
+      <c r="T18" s="34" t="n">
+        <f aca="false">COUNTA(T8:T17)</f>
+        <v>0</v>
+      </c>
+      <c r="U18" s="34" t="n">
+        <f aca="false">COUNTA(U8:U17)</f>
+        <v>0</v>
+      </c>
+      <c r="V18" s="34" t="n">
+        <f aca="false">COUNTA(V8:V17)</f>
+        <v>0</v>
+      </c>
+      <c r="W18" s="34" t="n">
+        <f aca="false">COUNTA(W8:W17)</f>
+        <v>0</v>
+      </c>
+      <c r="X18" s="34" t="n">
+        <f aca="false">COUNTA(X8:X17)</f>
+        <v>0</v>
+      </c>
+      <c r="Y18" s="34" t="n">
+        <f aca="false">COUNTA(Y8:Y17)</f>
+        <v>0</v>
+      </c>
+      <c r="Z18" s="34" t="n">
+        <f aca="false">COUNTA(Z8:Z17)</f>
+        <v>0</v>
+      </c>
+      <c r="AA18" s="34" t="n">
+        <f aca="false">COUNTA(AA8:AA17)</f>
+        <v>0</v>
+      </c>
+      <c r="AB18" s="34" t="n">
+        <f aca="false">COUNTA(AB8:AB17)</f>
+        <v>0</v>
+      </c>
+      <c r="AC18" s="34" t="n">
+        <f aca="false">COUNTA(AC8:AC17)</f>
+        <v>0</v>
+      </c>
+      <c r="AD18" s="34" t="n">
+        <f aca="false">COUNTA(AD8:AD17)</f>
+        <v>0</v>
+      </c>
+      <c r="AE18" s="34" t="n">
+        <f aca="false">COUNTA(AE8:AE17)</f>
+        <v>0</v>
+      </c>
+      <c r="AF18" s="34" t="n">
+        <f aca="false">COUNTA(AF8:AF17)</f>
+        <v>0</v>
+      </c>
+      <c r="AG18" s="34" t="n">
+        <f aca="false">COUNTA(AG8:AG17)</f>
+        <v>0</v>
+      </c>
+      <c r="AH18" s="34" t="n">
+        <f aca="false">COUNTA(AH8:AH17)</f>
+        <v>0</v>
+      </c>
+      <c r="AI18" s="34" t="n">
+        <f aca="false">COUNTA(AI8:AI17)</f>
+        <v>0</v>
+      </c>
+      <c r="AJ18" s="21" t="n">
+        <f aca="false">SUM(AJ8:AJ17)</f>
+        <v>0</v>
+      </c>
+      <c r="AK18" s="35"/>
+    </row>
+    <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="36" t="str">
+        <f aca="false">"МВГ «РОМБ» — особовий склад, осіб: "&amp;COUNTA(D20:D29)</f>
+        <v>МВГ «РОМБ» — особовий склад, осіб: 0</v>
+      </c>
+      <c r="B19" s="36"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="36"/>
+      <c r="E19" s="36"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="36"/>
+      <c r="H19" s="36"/>
+      <c r="I19" s="36"/>
+      <c r="J19" s="36"/>
+      <c r="K19" s="36"/>
+      <c r="L19" s="36"/>
+      <c r="M19" s="36"/>
+      <c r="N19" s="36"/>
+      <c r="O19" s="36"/>
+      <c r="P19" s="36"/>
+      <c r="Q19" s="36"/>
+      <c r="R19" s="36"/>
+      <c r="S19" s="36"/>
+      <c r="T19" s="36"/>
+      <c r="U19" s="36"/>
+      <c r="V19" s="36"/>
+      <c r="W19" s="36"/>
+      <c r="X19" s="36"/>
+      <c r="Y19" s="36"/>
+      <c r="Z19" s="36"/>
+      <c r="AA19" s="36"/>
+      <c r="AB19" s="36"/>
+      <c r="AC19" s="36"/>
+      <c r="AD19" s="36"/>
+      <c r="AE19" s="36"/>
+      <c r="AF19" s="36"/>
+      <c r="AG19" s="36"/>
+      <c r="AH19" s="36"/>
+      <c r="AI19" s="36"/>
+      <c r="AJ19" s="36"/>
+      <c r="AK19" s="36"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="31"/>
+      <c r="C20" s="31"/>
+      <c r="D20" s="31"/>
+      <c r="E20" s="31"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10"/>
+      <c r="L20" s="10"/>
+      <c r="M20" s="10"/>
+      <c r="N20" s="10"/>
+      <c r="O20" s="10"/>
+      <c r="P20" s="10"/>
+      <c r="Q20" s="10"/>
+      <c r="R20" s="10"/>
+      <c r="S20" s="10"/>
+      <c r="T20" s="10"/>
+      <c r="U20" s="10"/>
+      <c r="V20" s="10"/>
+      <c r="W20" s="10"/>
+      <c r="X20" s="10"/>
+      <c r="Y20" s="10"/>
+      <c r="Z20" s="10"/>
+      <c r="AA20" s="10"/>
+      <c r="AB20" s="10"/>
+      <c r="AC20" s="10"/>
+      <c r="AD20" s="10"/>
+      <c r="AE20" s="10"/>
+      <c r="AF20" s="10"/>
+      <c r="AG20" s="10"/>
+      <c r="AH20" s="10"/>
+      <c r="AI20" s="10"/>
+      <c r="AJ20" s="32" t="n">
+        <f aca="false">COUNTA(F20:AI20)</f>
+        <v>0</v>
+      </c>
+      <c r="AK20" s="33"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B21" s="31"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="10"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="10"/>
+      <c r="L21" s="10"/>
+      <c r="M21" s="10"/>
+      <c r="N21" s="10"/>
+      <c r="O21" s="10"/>
+      <c r="P21" s="10"/>
+      <c r="Q21" s="10"/>
+      <c r="R21" s="10"/>
+      <c r="S21" s="10"/>
+      <c r="T21" s="10"/>
+      <c r="U21" s="10"/>
+      <c r="V21" s="10"/>
+      <c r="W21" s="10"/>
+      <c r="X21" s="10"/>
+      <c r="Y21" s="10"/>
+      <c r="Z21" s="10"/>
+      <c r="AA21" s="10"/>
+      <c r="AB21" s="10"/>
+      <c r="AC21" s="10"/>
+      <c r="AD21" s="10"/>
+      <c r="AE21" s="10"/>
+      <c r="AF21" s="10"/>
+      <c r="AG21" s="10"/>
+      <c r="AH21" s="10"/>
+      <c r="AI21" s="10"/>
+      <c r="AJ21" s="32" t="n">
+        <f aca="false">COUNTA(F21:AI21)</f>
+        <v>0</v>
+      </c>
+      <c r="AK21" s="33"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" s="31"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="31"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="10"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="10"/>
+      <c r="L22" s="10"/>
+      <c r="M22" s="10"/>
+      <c r="N22" s="10"/>
+      <c r="O22" s="10"/>
+      <c r="P22" s="10"/>
+      <c r="Q22" s="10"/>
+      <c r="R22" s="10"/>
+      <c r="S22" s="10"/>
+      <c r="T22" s="10"/>
+      <c r="U22" s="10"/>
+      <c r="V22" s="10"/>
+      <c r="W22" s="10"/>
+      <c r="X22" s="10"/>
+      <c r="Y22" s="10"/>
+      <c r="Z22" s="10"/>
+      <c r="AA22" s="10"/>
+      <c r="AB22" s="10"/>
+      <c r="AC22" s="10"/>
+      <c r="AD22" s="10"/>
+      <c r="AE22" s="10"/>
+      <c r="AF22" s="10"/>
+      <c r="AG22" s="10"/>
+      <c r="AH22" s="10"/>
+      <c r="AI22" s="10"/>
+      <c r="AJ22" s="32" t="n">
+        <f aca="false">COUNTA(F22:AI22)</f>
+        <v>0</v>
+      </c>
+      <c r="AK22" s="33"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" s="31"/>
+      <c r="C23" s="31"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="31"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10"/>
+      <c r="P23" s="10"/>
+      <c r="Q23" s="10"/>
+      <c r="R23" s="10"/>
+      <c r="S23" s="10"/>
+      <c r="T23" s="10"/>
+      <c r="U23" s="10"/>
+      <c r="V23" s="10"/>
+      <c r="W23" s="10"/>
+      <c r="X23" s="10"/>
+      <c r="Y23" s="10"/>
+      <c r="Z23" s="10"/>
+      <c r="AA23" s="10"/>
+      <c r="AB23" s="10"/>
+      <c r="AC23" s="10"/>
+      <c r="AD23" s="10"/>
+      <c r="AE23" s="10"/>
+      <c r="AF23" s="10"/>
+      <c r="AG23" s="10"/>
+      <c r="AH23" s="10"/>
+      <c r="AI23" s="10"/>
+      <c r="AJ23" s="32" t="n">
+        <f aca="false">COUNTA(F23:AI23)</f>
+        <v>0</v>
+      </c>
+      <c r="AK23" s="33"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" s="31"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="31"/>
+      <c r="E24" s="31"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="10"/>
+      <c r="J24" s="10"/>
+      <c r="K24" s="10"/>
+      <c r="L24" s="10"/>
+      <c r="M24" s="10"/>
+      <c r="N24" s="10"/>
+      <c r="O24" s="10"/>
+      <c r="P24" s="10"/>
+      <c r="Q24" s="10"/>
+      <c r="R24" s="10"/>
+      <c r="S24" s="10"/>
+      <c r="T24" s="10"/>
+      <c r="U24" s="10"/>
+      <c r="V24" s="10"/>
+      <c r="W24" s="10"/>
+      <c r="X24" s="10"/>
+      <c r="Y24" s="10"/>
+      <c r="Z24" s="10"/>
+      <c r="AA24" s="10"/>
+      <c r="AB24" s="10"/>
+      <c r="AC24" s="10"/>
+      <c r="AD24" s="10"/>
+      <c r="AE24" s="10"/>
+      <c r="AF24" s="10"/>
+      <c r="AG24" s="10"/>
+      <c r="AH24" s="10"/>
+      <c r="AI24" s="10"/>
+      <c r="AJ24" s="32" t="n">
+        <f aca="false">COUNTA(F24:AI24)</f>
+        <v>0</v>
+      </c>
+      <c r="AK24" s="33"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B25" s="31"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="31"/>
+      <c r="E25" s="31"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="10"/>
+      <c r="K25" s="10"/>
+      <c r="L25" s="10"/>
+      <c r="M25" s="10"/>
+      <c r="N25" s="10"/>
+      <c r="O25" s="10"/>
+      <c r="P25" s="10"/>
+      <c r="Q25" s="10"/>
+      <c r="R25" s="10"/>
+      <c r="S25" s="10"/>
+      <c r="T25" s="10"/>
+      <c r="U25" s="10"/>
+      <c r="V25" s="10"/>
+      <c r="W25" s="10"/>
+      <c r="X25" s="10"/>
+      <c r="Y25" s="10"/>
+      <c r="Z25" s="10"/>
+      <c r="AA25" s="10"/>
+      <c r="AB25" s="10"/>
+      <c r="AC25" s="10"/>
+      <c r="AD25" s="10"/>
+      <c r="AE25" s="10"/>
+      <c r="AF25" s="10"/>
+      <c r="AG25" s="10"/>
+      <c r="AH25" s="10"/>
+      <c r="AI25" s="10"/>
+      <c r="AJ25" s="32" t="n">
+        <f aca="false">COUNTA(F25:AI25)</f>
+        <v>0</v>
+      </c>
+      <c r="AK25" s="33"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B26" s="31"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="10"/>
+      <c r="I26" s="10"/>
+      <c r="J26" s="10"/>
+      <c r="K26" s="10"/>
+      <c r="L26" s="10"/>
+      <c r="M26" s="10"/>
+      <c r="N26" s="10"/>
+      <c r="O26" s="10"/>
+      <c r="P26" s="10"/>
+      <c r="Q26" s="10"/>
+      <c r="R26" s="10"/>
+      <c r="S26" s="10"/>
+      <c r="T26" s="10"/>
+      <c r="U26" s="10"/>
+      <c r="V26" s="10"/>
+      <c r="W26" s="10"/>
+      <c r="X26" s="10"/>
+      <c r="Y26" s="10"/>
+      <c r="Z26" s="10"/>
+      <c r="AA26" s="10"/>
+      <c r="AB26" s="10"/>
+      <c r="AC26" s="10"/>
+      <c r="AD26" s="10"/>
+      <c r="AE26" s="10"/>
+      <c r="AF26" s="10"/>
+      <c r="AG26" s="10"/>
+      <c r="AH26" s="10"/>
+      <c r="AI26" s="10"/>
+      <c r="AJ26" s="32" t="n">
+        <f aca="false">COUNTA(F26:AI26)</f>
+        <v>0</v>
+      </c>
+      <c r="AK26" s="33"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B27" s="31"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="10"/>
+      <c r="J27" s="10"/>
+      <c r="K27" s="10"/>
+      <c r="L27" s="10"/>
+      <c r="M27" s="10"/>
+      <c r="N27" s="10"/>
+      <c r="O27" s="10"/>
+      <c r="P27" s="10"/>
+      <c r="Q27" s="10"/>
+      <c r="R27" s="10"/>
+      <c r="S27" s="10"/>
+      <c r="T27" s="10"/>
+      <c r="U27" s="10"/>
+      <c r="V27" s="10"/>
+      <c r="W27" s="10"/>
+      <c r="X27" s="10"/>
+      <c r="Y27" s="10"/>
+      <c r="Z27" s="10"/>
+      <c r="AA27" s="10"/>
+      <c r="AB27" s="10"/>
+      <c r="AC27" s="10"/>
+      <c r="AD27" s="10"/>
+      <c r="AE27" s="10"/>
+      <c r="AF27" s="10"/>
+      <c r="AG27" s="10"/>
+      <c r="AH27" s="10"/>
+      <c r="AI27" s="10"/>
+      <c r="AJ27" s="32" t="n">
+        <f aca="false">COUNTA(F27:AI27)</f>
+        <v>0</v>
+      </c>
+      <c r="AK27" s="33"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="B28" s="31"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="10"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="10"/>
+      <c r="L28" s="10"/>
+      <c r="M28" s="10"/>
+      <c r="N28" s="10"/>
+      <c r="O28" s="10"/>
+      <c r="P28" s="10"/>
+      <c r="Q28" s="10"/>
+      <c r="R28" s="10"/>
+      <c r="S28" s="10"/>
+      <c r="T28" s="10"/>
+      <c r="U28" s="10"/>
+      <c r="V28" s="10"/>
+      <c r="W28" s="10"/>
+      <c r="X28" s="10"/>
+      <c r="Y28" s="10"/>
+      <c r="Z28" s="10"/>
+      <c r="AA28" s="10"/>
+      <c r="AB28" s="10"/>
+      <c r="AC28" s="10"/>
+      <c r="AD28" s="10"/>
+      <c r="AE28" s="10"/>
+      <c r="AF28" s="10"/>
+      <c r="AG28" s="10"/>
+      <c r="AH28" s="10"/>
+      <c r="AI28" s="10"/>
+      <c r="AJ28" s="32" t="n">
+        <f aca="false">COUNTA(F28:AI28)</f>
+        <v>0</v>
+      </c>
+      <c r="AK28" s="33"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B29" s="31"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="31"/>
+      <c r="E29" s="31"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
+      <c r="L29" s="10"/>
+      <c r="M29" s="10"/>
+      <c r="N29" s="10"/>
+      <c r="O29" s="10"/>
+      <c r="P29" s="10"/>
+      <c r="Q29" s="10"/>
+      <c r="R29" s="10"/>
+      <c r="S29" s="10"/>
+      <c r="T29" s="10"/>
+      <c r="U29" s="10"/>
+      <c r="V29" s="10"/>
+      <c r="W29" s="10"/>
+      <c r="X29" s="10"/>
+      <c r="Y29" s="10"/>
+      <c r="Z29" s="10"/>
+      <c r="AA29" s="10"/>
+      <c r="AB29" s="10"/>
+      <c r="AC29" s="10"/>
+      <c r="AD29" s="10"/>
+      <c r="AE29" s="10"/>
+      <c r="AF29" s="10"/>
+      <c r="AG29" s="10"/>
+      <c r="AH29" s="10"/>
+      <c r="AI29" s="10"/>
+      <c r="AJ29" s="32" t="n">
+        <f aca="false">COUNTA(F29:AI29)</f>
+        <v>0</v>
+      </c>
+      <c r="AK29" s="33"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" s="18"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="34" t="n">
+        <f aca="false">COUNTA(F20:F29)</f>
+        <v>0</v>
+      </c>
+      <c r="G30" s="34" t="n">
+        <f aca="false">COUNTA(G20:G29)</f>
+        <v>0</v>
+      </c>
+      <c r="H30" s="34" t="n">
+        <f aca="false">COUNTA(H20:H29)</f>
+        <v>0</v>
+      </c>
+      <c r="I30" s="34" t="n">
+        <f aca="false">COUNTA(I20:I29)</f>
+        <v>0</v>
+      </c>
+      <c r="J30" s="34" t="n">
+        <f aca="false">COUNTA(J20:J29)</f>
+        <v>0</v>
+      </c>
+      <c r="K30" s="34" t="n">
+        <f aca="false">COUNTA(K20:K29)</f>
+        <v>0</v>
+      </c>
+      <c r="L30" s="34" t="n">
+        <f aca="false">COUNTA(L20:L29)</f>
+        <v>0</v>
+      </c>
+      <c r="M30" s="34" t="n">
+        <f aca="false">COUNTA(M20:M29)</f>
+        <v>0</v>
+      </c>
+      <c r="N30" s="34" t="n">
+        <f aca="false">COUNTA(N20:N29)</f>
+        <v>0</v>
+      </c>
+      <c r="O30" s="34" t="n">
+        <f aca="false">COUNTA(O20:O29)</f>
+        <v>0</v>
+      </c>
+      <c r="P30" s="34" t="n">
+        <f aca="false">COUNTA(P20:P29)</f>
+        <v>0</v>
+      </c>
+      <c r="Q30" s="34" t="n">
+        <f aca="false">COUNTA(Q20:Q29)</f>
+        <v>0</v>
+      </c>
+      <c r="R30" s="34" t="n">
+        <f aca="false">COUNTA(R20:R29)</f>
+        <v>0</v>
+      </c>
+      <c r="S30" s="34" t="n">
+        <f aca="false">COUNTA(S20:S29)</f>
+        <v>0</v>
+      </c>
+      <c r="T30" s="34" t="n">
+        <f aca="false">COUNTA(T20:T29)</f>
+        <v>0</v>
+      </c>
+      <c r="U30" s="34" t="n">
+        <f aca="false">COUNTA(U20:U29)</f>
+        <v>0</v>
+      </c>
+      <c r="V30" s="34" t="n">
+        <f aca="false">COUNTA(V20:V29)</f>
+        <v>0</v>
+      </c>
+      <c r="W30" s="34" t="n">
+        <f aca="false">COUNTA(W20:W29)</f>
+        <v>0</v>
+      </c>
+      <c r="X30" s="34" t="n">
+        <f aca="false">COUNTA(X20:X29)</f>
+        <v>0</v>
+      </c>
+      <c r="Y30" s="34" t="n">
+        <f aca="false">COUNTA(Y20:Y29)</f>
+        <v>0</v>
+      </c>
+      <c r="Z30" s="34" t="n">
+        <f aca="false">COUNTA(Z20:Z29)</f>
+        <v>0</v>
+      </c>
+      <c r="AA30" s="34" t="n">
+        <f aca="false">COUNTA(AA20:AA29)</f>
+        <v>0</v>
+      </c>
+      <c r="AB30" s="34" t="n">
+        <f aca="false">COUNTA(AB20:AB29)</f>
+        <v>0</v>
+      </c>
+      <c r="AC30" s="34" t="n">
+        <f aca="false">COUNTA(AC20:AC29)</f>
+        <v>0</v>
+      </c>
+      <c r="AD30" s="34" t="n">
+        <f aca="false">COUNTA(AD20:AD29)</f>
+        <v>0</v>
+      </c>
+      <c r="AE30" s="34" t="n">
+        <f aca="false">COUNTA(AE20:AE29)</f>
+        <v>0</v>
+      </c>
+      <c r="AF30" s="34" t="n">
+        <f aca="false">COUNTA(AF20:AF29)</f>
+        <v>0</v>
+      </c>
+      <c r="AG30" s="34" t="n">
+        <f aca="false">COUNTA(AG20:AG29)</f>
+        <v>0</v>
+      </c>
+      <c r="AH30" s="34" t="n">
+        <f aca="false">COUNTA(AH20:AH29)</f>
+        <v>0</v>
+      </c>
+      <c r="AI30" s="34" t="n">
+        <f aca="false">COUNTA(AI20:AI29)</f>
+        <v>0</v>
+      </c>
+      <c r="AJ30" s="21" t="n">
+        <f aca="false">SUM(AJ20:AJ29)</f>
+        <v>0</v>
+      </c>
+      <c r="AK30" s="35"/>
+    </row>
+    <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="37" t="str">
+        <f aca="false">"МВГ «ДАЧА» — особовий склад, осіб: "&amp;COUNTA(D32:D41)</f>
+        <v>МВГ «ДАЧА» — особовий склад, осіб: 0</v>
+      </c>
+      <c r="B31" s="37"/>
+      <c r="C31" s="37"/>
+      <c r="D31" s="37"/>
+      <c r="E31" s="37"/>
+      <c r="F31" s="37"/>
+      <c r="G31" s="37"/>
+      <c r="H31" s="37"/>
+      <c r="I31" s="37"/>
+      <c r="J31" s="37"/>
+      <c r="K31" s="37"/>
+      <c r="L31" s="37"/>
+      <c r="M31" s="37"/>
+      <c r="N31" s="37"/>
+      <c r="O31" s="37"/>
+      <c r="P31" s="37"/>
+      <c r="Q31" s="37"/>
+      <c r="R31" s="37"/>
+      <c r="S31" s="37"/>
+      <c r="T31" s="37"/>
+      <c r="U31" s="37"/>
+      <c r="V31" s="37"/>
+      <c r="W31" s="37"/>
+      <c r="X31" s="37"/>
+      <c r="Y31" s="37"/>
+      <c r="Z31" s="37"/>
+      <c r="AA31" s="37"/>
+      <c r="AB31" s="37"/>
+      <c r="AC31" s="37"/>
+      <c r="AD31" s="37"/>
+      <c r="AE31" s="37"/>
+      <c r="AF31" s="37"/>
+      <c r="AG31" s="37"/>
+      <c r="AH31" s="37"/>
+      <c r="AI31" s="37"/>
+      <c r="AJ31" s="37"/>
+      <c r="AK31" s="37"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B32" s="31"/>
+      <c r="C32" s="31"/>
+      <c r="D32" s="31"/>
+      <c r="E32" s="31"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="10"/>
+      <c r="I32" s="10"/>
+      <c r="J32" s="10"/>
+      <c r="K32" s="10"/>
+      <c r="L32" s="10"/>
+      <c r="M32" s="10"/>
+      <c r="N32" s="10"/>
+      <c r="O32" s="10"/>
+      <c r="P32" s="10"/>
+      <c r="Q32" s="10"/>
+      <c r="R32" s="10"/>
+      <c r="S32" s="10"/>
+      <c r="T32" s="10"/>
+      <c r="U32" s="10"/>
+      <c r="V32" s="10"/>
+      <c r="W32" s="10"/>
+      <c r="X32" s="10"/>
+      <c r="Y32" s="10"/>
+      <c r="Z32" s="10"/>
+      <c r="AA32" s="10"/>
+      <c r="AB32" s="10"/>
+      <c r="AC32" s="10"/>
+      <c r="AD32" s="10"/>
+      <c r="AE32" s="10"/>
+      <c r="AF32" s="10"/>
+      <c r="AG32" s="10"/>
+      <c r="AH32" s="10"/>
+      <c r="AI32" s="10"/>
+      <c r="AJ32" s="32" t="n">
+        <f aca="false">COUNTA(F32:AI32)</f>
+        <v>0</v>
+      </c>
+      <c r="AK32" s="33"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B33" s="31"/>
+      <c r="C33" s="31"/>
+      <c r="D33" s="31"/>
+      <c r="E33" s="31"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="10"/>
+      <c r="H33" s="10"/>
+      <c r="I33" s="10"/>
+      <c r="J33" s="10"/>
+      <c r="K33" s="10"/>
+      <c r="L33" s="10"/>
+      <c r="M33" s="10"/>
+      <c r="N33" s="10"/>
+      <c r="O33" s="10"/>
+      <c r="P33" s="10"/>
+      <c r="Q33" s="10"/>
+      <c r="R33" s="10"/>
+      <c r="S33" s="10"/>
+      <c r="T33" s="10"/>
+      <c r="U33" s="10"/>
+      <c r="V33" s="10"/>
+      <c r="W33" s="10"/>
+      <c r="X33" s="10"/>
+      <c r="Y33" s="10"/>
+      <c r="Z33" s="10"/>
+      <c r="AA33" s="10"/>
+      <c r="AB33" s="10"/>
+      <c r="AC33" s="10"/>
+      <c r="AD33" s="10"/>
+      <c r="AE33" s="10"/>
+      <c r="AF33" s="10"/>
+      <c r="AG33" s="10"/>
+      <c r="AH33" s="10"/>
+      <c r="AI33" s="10"/>
+      <c r="AJ33" s="32" t="n">
+        <f aca="false">COUNTA(F33:AI33)</f>
+        <v>0</v>
+      </c>
+      <c r="AK33" s="33"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B34" s="31"/>
+      <c r="C34" s="31"/>
+      <c r="D34" s="31"/>
+      <c r="E34" s="31"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="10"/>
+      <c r="H34" s="10"/>
+      <c r="I34" s="10"/>
+      <c r="J34" s="10"/>
+      <c r="K34" s="10"/>
+      <c r="L34" s="10"/>
+      <c r="M34" s="10"/>
+      <c r="N34" s="10"/>
+      <c r="O34" s="10"/>
+      <c r="P34" s="10"/>
+      <c r="Q34" s="10"/>
+      <c r="R34" s="10"/>
+      <c r="S34" s="10"/>
+      <c r="T34" s="10"/>
+      <c r="U34" s="10"/>
+      <c r="V34" s="10"/>
+      <c r="W34" s="10"/>
+      <c r="X34" s="10"/>
+      <c r="Y34" s="10"/>
+      <c r="Z34" s="10"/>
+      <c r="AA34" s="10"/>
+      <c r="AB34" s="10"/>
+      <c r="AC34" s="10"/>
+      <c r="AD34" s="10"/>
+      <c r="AE34" s="10"/>
+      <c r="AF34" s="10"/>
+      <c r="AG34" s="10"/>
+      <c r="AH34" s="10"/>
+      <c r="AI34" s="10"/>
+      <c r="AJ34" s="32" t="n">
+        <f aca="false">COUNTA(F34:AI34)</f>
+        <v>0</v>
+      </c>
+      <c r="AK34" s="33"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B35" s="31"/>
+      <c r="C35" s="31"/>
+      <c r="D35" s="31"/>
+      <c r="E35" s="31"/>
+      <c r="F35" s="10"/>
+      <c r="G35" s="10"/>
+      <c r="H35" s="10"/>
+      <c r="I35" s="10"/>
+      <c r="J35" s="10"/>
+      <c r="K35" s="10"/>
+      <c r="L35" s="10"/>
+      <c r="M35" s="10"/>
+      <c r="N35" s="10"/>
+      <c r="O35" s="10"/>
+      <c r="P35" s="10"/>
+      <c r="Q35" s="10"/>
+      <c r="R35" s="10"/>
+      <c r="S35" s="10"/>
+      <c r="T35" s="10"/>
+      <c r="U35" s="10"/>
+      <c r="V35" s="10"/>
+      <c r="W35" s="10"/>
+      <c r="X35" s="10"/>
+      <c r="Y35" s="10"/>
+      <c r="Z35" s="10"/>
+      <c r="AA35" s="10"/>
+      <c r="AB35" s="10"/>
+      <c r="AC35" s="10"/>
+      <c r="AD35" s="10"/>
+      <c r="AE35" s="10"/>
+      <c r="AF35" s="10"/>
+      <c r="AG35" s="10"/>
+      <c r="AH35" s="10"/>
+      <c r="AI35" s="10"/>
+      <c r="AJ35" s="32" t="n">
+        <f aca="false">COUNTA(F35:AI35)</f>
+        <v>0</v>
+      </c>
+      <c r="AK35" s="33"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B36" s="31"/>
+      <c r="C36" s="31"/>
+      <c r="D36" s="31"/>
+      <c r="E36" s="31"/>
+      <c r="F36" s="10"/>
+      <c r="G36" s="10"/>
+      <c r="H36" s="10"/>
+      <c r="I36" s="10"/>
+      <c r="J36" s="10"/>
+      <c r="K36" s="10"/>
+      <c r="L36" s="10"/>
+      <c r="M36" s="10"/>
+      <c r="N36" s="10"/>
+      <c r="O36" s="10"/>
+      <c r="P36" s="10"/>
+      <c r="Q36" s="10"/>
+      <c r="R36" s="10"/>
+      <c r="S36" s="10"/>
+      <c r="T36" s="10"/>
+      <c r="U36" s="10"/>
+      <c r="V36" s="10"/>
+      <c r="W36" s="10"/>
+      <c r="X36" s="10"/>
+      <c r="Y36" s="10"/>
+      <c r="Z36" s="10"/>
+      <c r="AA36" s="10"/>
+      <c r="AB36" s="10"/>
+      <c r="AC36" s="10"/>
+      <c r="AD36" s="10"/>
+      <c r="AE36" s="10"/>
+      <c r="AF36" s="10"/>
+      <c r="AG36" s="10"/>
+      <c r="AH36" s="10"/>
+      <c r="AI36" s="10"/>
+      <c r="AJ36" s="32" t="n">
+        <f aca="false">COUNTA(F36:AI36)</f>
+        <v>0</v>
+      </c>
+      <c r="AK36" s="33"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B37" s="31"/>
+      <c r="C37" s="31"/>
+      <c r="D37" s="31"/>
+      <c r="E37" s="31"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="10"/>
+      <c r="H37" s="10"/>
+      <c r="I37" s="10"/>
+      <c r="J37" s="10"/>
+      <c r="K37" s="10"/>
+      <c r="L37" s="10"/>
+      <c r="M37" s="10"/>
+      <c r="N37" s="10"/>
+      <c r="O37" s="10"/>
+      <c r="P37" s="10"/>
+      <c r="Q37" s="10"/>
+      <c r="R37" s="10"/>
+      <c r="S37" s="10"/>
+      <c r="T37" s="10"/>
+      <c r="U37" s="10"/>
+      <c r="V37" s="10"/>
+      <c r="W37" s="10"/>
+      <c r="X37" s="10"/>
+      <c r="Y37" s="10"/>
+      <c r="Z37" s="10"/>
+      <c r="AA37" s="10"/>
+      <c r="AB37" s="10"/>
+      <c r="AC37" s="10"/>
+      <c r="AD37" s="10"/>
+      <c r="AE37" s="10"/>
+      <c r="AF37" s="10"/>
+      <c r="AG37" s="10"/>
+      <c r="AH37" s="10"/>
+      <c r="AI37" s="10"/>
+      <c r="AJ37" s="32" t="n">
+        <f aca="false">COUNTA(F37:AI37)</f>
+        <v>0</v>
+      </c>
+      <c r="AK37" s="33"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B38" s="31"/>
+      <c r="C38" s="31"/>
+      <c r="D38" s="31"/>
+      <c r="E38" s="31"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="10"/>
+      <c r="H38" s="10"/>
+      <c r="I38" s="10"/>
+      <c r="J38" s="10"/>
+      <c r="K38" s="10"/>
+      <c r="L38" s="10"/>
+      <c r="M38" s="10"/>
+      <c r="N38" s="10"/>
+      <c r="O38" s="10"/>
+      <c r="P38" s="10"/>
+      <c r="Q38" s="10"/>
+      <c r="R38" s="10"/>
+      <c r="S38" s="10"/>
+      <c r="T38" s="10"/>
+      <c r="U38" s="10"/>
+      <c r="V38" s="10"/>
+      <c r="W38" s="10"/>
+      <c r="X38" s="10"/>
+      <c r="Y38" s="10"/>
+      <c r="Z38" s="10"/>
+      <c r="AA38" s="10"/>
+      <c r="AB38" s="10"/>
+      <c r="AC38" s="10"/>
+      <c r="AD38" s="10"/>
+      <c r="AE38" s="10"/>
+      <c r="AF38" s="10"/>
+      <c r="AG38" s="10"/>
+      <c r="AH38" s="10"/>
+      <c r="AI38" s="10"/>
+      <c r="AJ38" s="32" t="n">
+        <f aca="false">COUNTA(F38:AI38)</f>
+        <v>0</v>
+      </c>
+      <c r="AK38" s="33"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B39" s="31"/>
+      <c r="C39" s="31"/>
+      <c r="D39" s="31"/>
+      <c r="E39" s="31"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="10"/>
+      <c r="H39" s="10"/>
+      <c r="I39" s="10"/>
+      <c r="J39" s="10"/>
+      <c r="K39" s="10"/>
+      <c r="L39" s="10"/>
+      <c r="M39" s="10"/>
+      <c r="N39" s="10"/>
+      <c r="O39" s="10"/>
+      <c r="P39" s="10"/>
+      <c r="Q39" s="10"/>
+      <c r="R39" s="10"/>
+      <c r="S39" s="10"/>
+      <c r="T39" s="10"/>
+      <c r="U39" s="10"/>
+      <c r="V39" s="10"/>
+      <c r="W39" s="10"/>
+      <c r="X39" s="10"/>
+      <c r="Y39" s="10"/>
+      <c r="Z39" s="10"/>
+      <c r="AA39" s="10"/>
+      <c r="AB39" s="10"/>
+      <c r="AC39" s="10"/>
+      <c r="AD39" s="10"/>
+      <c r="AE39" s="10"/>
+      <c r="AF39" s="10"/>
+      <c r="AG39" s="10"/>
+      <c r="AH39" s="10"/>
+      <c r="AI39" s="10"/>
+      <c r="AJ39" s="32" t="n">
+        <f aca="false">COUNTA(F39:AI39)</f>
+        <v>0</v>
+      </c>
+      <c r="AK39" s="33"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="B40" s="31"/>
+      <c r="C40" s="31"/>
+      <c r="D40" s="31"/>
+      <c r="E40" s="31"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="10"/>
+      <c r="J40" s="10"/>
+      <c r="K40" s="10"/>
+      <c r="L40" s="10"/>
+      <c r="M40" s="10"/>
+      <c r="N40" s="10"/>
+      <c r="O40" s="10"/>
+      <c r="P40" s="10"/>
+      <c r="Q40" s="10"/>
+      <c r="R40" s="10"/>
+      <c r="S40" s="10"/>
+      <c r="T40" s="10"/>
+      <c r="U40" s="10"/>
+      <c r="V40" s="10"/>
+      <c r="W40" s="10"/>
+      <c r="X40" s="10"/>
+      <c r="Y40" s="10"/>
+      <c r="Z40" s="10"/>
+      <c r="AA40" s="10"/>
+      <c r="AB40" s="10"/>
+      <c r="AC40" s="10"/>
+      <c r="AD40" s="10"/>
+      <c r="AE40" s="10"/>
+      <c r="AF40" s="10"/>
+      <c r="AG40" s="10"/>
+      <c r="AH40" s="10"/>
+      <c r="AI40" s="10"/>
+      <c r="AJ40" s="32" t="n">
+        <f aca="false">COUNTA(F40:AI40)</f>
+        <v>0</v>
+      </c>
+      <c r="AK40" s="33"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B41" s="31"/>
+      <c r="C41" s="31"/>
+      <c r="D41" s="31"/>
+      <c r="E41" s="31"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="I41" s="10"/>
+      <c r="J41" s="10"/>
+      <c r="K41" s="10"/>
+      <c r="L41" s="10"/>
+      <c r="M41" s="10"/>
+      <c r="N41" s="10"/>
+      <c r="O41" s="10"/>
+      <c r="P41" s="10"/>
+      <c r="Q41" s="10"/>
+      <c r="R41" s="10"/>
+      <c r="S41" s="10"/>
+      <c r="T41" s="10"/>
+      <c r="U41" s="10"/>
+      <c r="V41" s="10"/>
+      <c r="W41" s="10"/>
+      <c r="X41" s="10"/>
+      <c r="Y41" s="10"/>
+      <c r="Z41" s="10"/>
+      <c r="AA41" s="10"/>
+      <c r="AB41" s="10"/>
+      <c r="AC41" s="10"/>
+      <c r="AD41" s="10"/>
+      <c r="AE41" s="10"/>
+      <c r="AF41" s="10"/>
+      <c r="AG41" s="10"/>
+      <c r="AH41" s="10"/>
+      <c r="AI41" s="10"/>
+      <c r="AJ41" s="32" t="n">
+        <f aca="false">COUNTA(F41:AI41)</f>
+        <v>0</v>
+      </c>
+      <c r="AK41" s="33"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B42" s="18"/>
+      <c r="C42" s="18"/>
+      <c r="D42" s="18"/>
+      <c r="E42" s="18"/>
+      <c r="F42" s="34" t="n">
+        <f aca="false">COUNTA(F32:F41)</f>
+        <v>0</v>
+      </c>
+      <c r="G42" s="34" t="n">
+        <f aca="false">COUNTA(G32:G41)</f>
+        <v>0</v>
+      </c>
+      <c r="H42" s="34" t="n">
+        <f aca="false">COUNTA(H32:H41)</f>
+        <v>0</v>
+      </c>
+      <c r="I42" s="34" t="n">
+        <f aca="false">COUNTA(I32:I41)</f>
+        <v>0</v>
+      </c>
+      <c r="J42" s="34" t="n">
+        <f aca="false">COUNTA(J32:J41)</f>
+        <v>0</v>
+      </c>
+      <c r="K42" s="34" t="n">
+        <f aca="false">COUNTA(K32:K41)</f>
+        <v>0</v>
+      </c>
+      <c r="L42" s="34" t="n">
+        <f aca="false">COUNTA(L32:L41)</f>
+        <v>0</v>
+      </c>
+      <c r="M42" s="34" t="n">
+        <f aca="false">COUNTA(M32:M41)</f>
+        <v>0</v>
+      </c>
+      <c r="N42" s="34" t="n">
+        <f aca="false">COUNTA(N32:N41)</f>
+        <v>0</v>
+      </c>
+      <c r="O42" s="34" t="n">
+        <f aca="false">COUNTA(O32:O41)</f>
+        <v>0</v>
+      </c>
+      <c r="P42" s="34" t="n">
+        <f aca="false">COUNTA(P32:P41)</f>
+        <v>0</v>
+      </c>
+      <c r="Q42" s="34" t="n">
+        <f aca="false">COUNTA(Q32:Q41)</f>
+        <v>0</v>
+      </c>
+      <c r="R42" s="34" t="n">
+        <f aca="false">COUNTA(R32:R41)</f>
+        <v>0</v>
+      </c>
+      <c r="S42" s="34" t="n">
+        <f aca="false">COUNTA(S32:S41)</f>
+        <v>0</v>
+      </c>
+      <c r="T42" s="34" t="n">
+        <f aca="false">COUNTA(T32:T41)</f>
+        <v>0</v>
+      </c>
+      <c r="U42" s="34" t="n">
+        <f aca="false">COUNTA(U32:U41)</f>
+        <v>0</v>
+      </c>
+      <c r="V42" s="34" t="n">
+        <f aca="false">COUNTA(V32:V41)</f>
+        <v>0</v>
+      </c>
+      <c r="W42" s="34" t="n">
+        <f aca="false">COUNTA(W32:W41)</f>
+        <v>0</v>
+      </c>
+      <c r="X42" s="34" t="n">
+        <f aca="false">COUNTA(X32:X41)</f>
+        <v>0</v>
+      </c>
+      <c r="Y42" s="34" t="n">
+        <f aca="false">COUNTA(Y32:Y41)</f>
+        <v>0</v>
+      </c>
+      <c r="Z42" s="34" t="n">
+        <f aca="false">COUNTA(Z32:Z41)</f>
+        <v>0</v>
+      </c>
+      <c r="AA42" s="34" t="n">
+        <f aca="false">COUNTA(AA32:AA41)</f>
+        <v>0</v>
+      </c>
+      <c r="AB42" s="34" t="n">
+        <f aca="false">COUNTA(AB32:AB41)</f>
+        <v>0</v>
+      </c>
+      <c r="AC42" s="34" t="n">
+        <f aca="false">COUNTA(AC32:AC41)</f>
+        <v>0</v>
+      </c>
+      <c r="AD42" s="34" t="n">
+        <f aca="false">COUNTA(AD32:AD41)</f>
+        <v>0</v>
+      </c>
+      <c r="AE42" s="34" t="n">
+        <f aca="false">COUNTA(AE32:AE41)</f>
+        <v>0</v>
+      </c>
+      <c r="AF42" s="34" t="n">
+        <f aca="false">COUNTA(AF32:AF41)</f>
+        <v>0</v>
+      </c>
+      <c r="AG42" s="34" t="n">
+        <f aca="false">COUNTA(AG32:AG41)</f>
+        <v>0</v>
+      </c>
+      <c r="AH42" s="34" t="n">
+        <f aca="false">COUNTA(AH32:AH41)</f>
+        <v>0</v>
+      </c>
+      <c r="AI42" s="34" t="n">
+        <f aca="false">COUNTA(AI32:AI41)</f>
+        <v>0</v>
+      </c>
+      <c r="AJ42" s="21" t="n">
+        <f aca="false">SUM(AJ32:AJ41)</f>
+        <v>0</v>
+      </c>
+      <c r="AK42" s="35"/>
+    </row>
+    <row r="43" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B43" s="15"/>
+      <c r="C43" s="15"/>
+      <c r="D43" s="15"/>
+      <c r="E43" s="15"/>
+      <c r="F43" s="38" t="n">
+        <f aca="false">F18+F30+F42</f>
+        <v>0</v>
+      </c>
+      <c r="G43" s="38" t="n">
+        <f aca="false">G18+G30+G42</f>
+        <v>0</v>
+      </c>
+      <c r="H43" s="38" t="n">
+        <f aca="false">H18+H30+H42</f>
+        <v>0</v>
+      </c>
+      <c r="I43" s="38" t="n">
+        <f aca="false">I18+I30+I42</f>
+        <v>0</v>
+      </c>
+      <c r="J43" s="38" t="n">
+        <f aca="false">J18+J30+J42</f>
+        <v>0</v>
+      </c>
+      <c r="K43" s="38" t="n">
+        <f aca="false">K18+K30+K42</f>
+        <v>0</v>
+      </c>
+      <c r="L43" s="38" t="n">
+        <f aca="false">L18+L30+L42</f>
+        <v>0</v>
+      </c>
+      <c r="M43" s="38" t="n">
+        <f aca="false">M18+M30+M42</f>
+        <v>0</v>
+      </c>
+      <c r="N43" s="38" t="n">
+        <f aca="false">N18+N30+N42</f>
+        <v>0</v>
+      </c>
+      <c r="O43" s="38" t="n">
+        <f aca="false">O18+O30+O42</f>
+        <v>0</v>
+      </c>
+      <c r="P43" s="38" t="n">
+        <f aca="false">P18+P30+P42</f>
+        <v>0</v>
+      </c>
+      <c r="Q43" s="38" t="n">
+        <f aca="false">Q18+Q30+Q42</f>
+        <v>0</v>
+      </c>
+      <c r="R43" s="38" t="n">
+        <f aca="false">R18+R30+R42</f>
+        <v>0</v>
+      </c>
+      <c r="S43" s="38" t="n">
+        <f aca="false">S18+S30+S42</f>
+        <v>0</v>
+      </c>
+      <c r="T43" s="38" t="n">
+        <f aca="false">T18+T30+T42</f>
+        <v>0</v>
+      </c>
+      <c r="U43" s="38" t="n">
+        <f aca="false">U18+U30+U42</f>
+        <v>0</v>
+      </c>
+      <c r="V43" s="38" t="n">
+        <f aca="false">V18+V30+V42</f>
+        <v>0</v>
+      </c>
+      <c r="W43" s="38" t="n">
+        <f aca="false">W18+W30+W42</f>
+        <v>0</v>
+      </c>
+      <c r="X43" s="38" t="n">
+        <f aca="false">X18+X30+X42</f>
+        <v>0</v>
+      </c>
+      <c r="Y43" s="38" t="n">
+        <f aca="false">Y18+Y30+Y42</f>
+        <v>0</v>
+      </c>
+      <c r="Z43" s="38" t="n">
+        <f aca="false">Z18+Z30+Z42</f>
+        <v>0</v>
+      </c>
+      <c r="AA43" s="38" t="n">
+        <f aca="false">AA18+AA30+AA42</f>
+        <v>0</v>
+      </c>
+      <c r="AB43" s="38" t="n">
+        <f aca="false">AB18+AB30+AB42</f>
+        <v>0</v>
+      </c>
+      <c r="AC43" s="38" t="n">
+        <f aca="false">AC18+AC30+AC42</f>
+        <v>0</v>
+      </c>
+      <c r="AD43" s="38" t="n">
+        <f aca="false">AD18+AD30+AD42</f>
+        <v>0</v>
+      </c>
+      <c r="AE43" s="38" t="n">
+        <f aca="false">AE18+AE30+AE42</f>
+        <v>0</v>
+      </c>
+      <c r="AF43" s="38" t="n">
+        <f aca="false">AF18+AF30+AF42</f>
+        <v>0</v>
+      </c>
+      <c r="AG43" s="38" t="n">
+        <f aca="false">AG18+AG30+AG42</f>
+        <v>0</v>
+      </c>
+      <c r="AH43" s="38" t="n">
+        <f aca="false">AH18+AH30+AH42</f>
+        <v>0</v>
+      </c>
+      <c r="AI43" s="38" t="n">
+        <f aca="false">AI18+AI30+AI42</f>
+        <v>0</v>
+      </c>
+      <c r="AJ43" s="16" t="n">
+        <f aca="false">AJ18+AJ30+AJ42</f>
+        <v>0</v>
+      </c>
+      <c r="AK43" s="39"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="22" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="23" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="23" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="23" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="23" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="23" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="24" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="B52" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="C52" s="27" t="s">
+        <v>45</v>
+      </c>
+      <c r="D52" s="27" t="s">
+        <v>46</v>
+      </c>
+      <c r="E52" s="27" t="s">
+        <v>47</v>
+      </c>
+      <c r="F52" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="G52" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="H52" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="I52" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="J52" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="K52" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="L52" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="M52" s="25"/>
+      <c r="N52" s="25"/>
+      <c r="O52" s="25"/>
+      <c r="P52" s="25"/>
+      <c r="Q52" s="25"/>
+      <c r="R52" s="25"/>
+      <c r="S52" s="25"/>
+      <c r="T52" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="U52" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="V52" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="W52" s="25"/>
+      <c r="X52" s="25"/>
+      <c r="Y52" s="25"/>
+      <c r="Z52" s="25"/>
+      <c r="AA52" s="25"/>
+      <c r="AB52" s="25"/>
+      <c r="AC52" s="25"/>
+      <c r="AD52" s="25"/>
+      <c r="AE52" s="25"/>
+      <c r="AF52" s="25"/>
+      <c r="AG52" s="25"/>
+      <c r="AH52" s="25"/>
+      <c r="AI52" s="25"/>
+      <c r="AJ52" s="25" t="n">
+        <f aca="false">COUNTA(F52:AI52)</f>
+        <v>10</v>
+      </c>
+      <c r="AK52" s="40" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="28" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="17">
+    <mergeCell ref="A1:AK1"/>
+    <mergeCell ref="A2:AK2"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="C4:C6"/>
+    <mergeCell ref="D4:D6"/>
+    <mergeCell ref="E4:E6"/>
+    <mergeCell ref="F4:AI4"/>
+    <mergeCell ref="AJ4:AJ6"/>
+    <mergeCell ref="AK4:AK6"/>
+    <mergeCell ref="A7:AK7"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A19:AK19"/>
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A31:AK31"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A43:E43"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B8:B17 B20:B29 B32:B41" type="list">
+      <formula1>"Старший групи,Кулеметник,Навідник,Стрілець,Спостерігач,Оператор,Водій"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C8:C17 C20:C29 C32:C41" type="list">
+      <formula1>"солдат,старший солдат,молодший сержант,сержант,старший сержант,головний сержант,штаб-сержант,майстер-сержант,молодший лейтенант,лейтенант,старший лейтенант,капітан,майор"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
+  <pageMargins left="0.3" right="0.3" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -2807,25 +5463,29 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="29" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
+      <c r="A1" s="41" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
     </row>
     <row r="3" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>10</v>
@@ -2840,10 +5500,10 @@
         <v>13</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>15</v>
@@ -2852,30 +5512,36 @@
         <v>16</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>30</v>
+        <v>54</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="30" t="s">
+      <c r="A4" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="31" t="n">
+      <c r="B4" s="43" t="n">
         <f aca="false">'Щоденний облік'!D36</f>
         <v>0</v>
       </c>
-      <c r="C4" s="31" t="n">
+      <c r="C4" s="43" t="n">
         <f aca="false">'Щоденний облік'!E36</f>
         <v>0</v>
       </c>
-      <c r="D4" s="31" t="n">
+      <c r="D4" s="43" t="n">
         <f aca="false">'Щоденний облік'!F36</f>
         <v>0</v>
       </c>
-      <c r="E4" s="32" t="n">
+      <c r="E4" s="44" t="n">
         <f aca="false">'Щоденний облік'!G36</f>
         <v>0</v>
       </c>
-      <c r="F4" s="33" t="n">
+      <c r="F4" s="45" t="n">
         <f aca="false">IF($E$7=0,0,E4/$E$7)</f>
         <v>0</v>
       </c>
@@ -2883,7 +5549,7 @@
         <f aca="false">COUNTIF('Щоденний облік'!$G$6:$G$35,"&gt;0")</f>
         <v>0</v>
       </c>
-      <c r="H4" s="34" t="n">
+      <c r="H4" s="46" t="n">
         <f aca="false">E4/COUNT('Щоденний облік'!$B$6:$B$35)</f>
         <v>0</v>
       </c>
@@ -2895,28 +5561,36 @@
         <f aca="false">IF(I4=0,"—",INDEX('Щоденний облік'!$B$6:$B$35,MATCH(I4,'Щоденний облік'!$G$6:$G$35,0)))</f>
         <v>—</v>
       </c>
+      <c r="K4" s="8" t="n">
+        <f aca="false">COUNTA('Склад МВГ'!D8:D17)</f>
+        <v>0</v>
+      </c>
+      <c r="L4" s="43" t="n">
+        <f aca="false">'Склад МВГ'!AJ18</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="35" t="s">
+      <c r="A5" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="31" t="n">
+      <c r="B5" s="43" t="n">
         <f aca="false">'Щоденний облік'!H36</f>
         <v>0</v>
       </c>
-      <c r="C5" s="31" t="n">
+      <c r="C5" s="43" t="n">
         <f aca="false">'Щоденний облік'!I36</f>
         <v>0</v>
       </c>
-      <c r="D5" s="31" t="n">
+      <c r="D5" s="43" t="n">
         <f aca="false">'Щоденний облік'!J36</f>
         <v>0</v>
       </c>
-      <c r="E5" s="32" t="n">
+      <c r="E5" s="44" t="n">
         <f aca="false">'Щоденний облік'!K36</f>
         <v>0</v>
       </c>
-      <c r="F5" s="33" t="n">
+      <c r="F5" s="45" t="n">
         <f aca="false">IF($E$7=0,0,E5/$E$7)</f>
         <v>0</v>
       </c>
@@ -2924,7 +5598,7 @@
         <f aca="false">COUNTIF('Щоденний облік'!$K$6:$K$35,"&gt;0")</f>
         <v>0</v>
       </c>
-      <c r="H5" s="34" t="n">
+      <c r="H5" s="46" t="n">
         <f aca="false">E5/COUNT('Щоденний облік'!$B$6:$B$35)</f>
         <v>0</v>
       </c>
@@ -2936,28 +5610,36 @@
         <f aca="false">IF(I5=0,"—",INDEX('Щоденний облік'!$B$6:$B$35,MATCH(I5,'Щоденний облік'!$K$6:$K$35,0)))</f>
         <v>—</v>
       </c>
+      <c r="K5" s="8" t="n">
+        <f aca="false">COUNTA('Склад МВГ'!D20:D29)</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="43" t="n">
+        <f aca="false">'Склад МВГ'!AJ30</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="36" t="s">
+      <c r="A6" s="48" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="31" t="n">
+      <c r="B6" s="43" t="n">
         <f aca="false">'Щоденний облік'!L36</f>
         <v>0</v>
       </c>
-      <c r="C6" s="31" t="n">
+      <c r="C6" s="43" t="n">
         <f aca="false">'Щоденний облік'!M36</f>
         <v>0</v>
       </c>
-      <c r="D6" s="31" t="n">
+      <c r="D6" s="43" t="n">
         <f aca="false">'Щоденний облік'!N36</f>
         <v>0</v>
       </c>
-      <c r="E6" s="32" t="n">
+      <c r="E6" s="44" t="n">
         <f aca="false">'Щоденний облік'!O36</f>
         <v>0</v>
       </c>
-      <c r="F6" s="33" t="n">
+      <c r="F6" s="45" t="n">
         <f aca="false">IF($E$7=0,0,E6/$E$7)</f>
         <v>0</v>
       </c>
@@ -2965,7 +5647,7 @@
         <f aca="false">COUNTIF('Щоденний облік'!$O$6:$O$35,"&gt;0")</f>
         <v>0</v>
       </c>
-      <c r="H6" s="34" t="n">
+      <c r="H6" s="46" t="n">
         <f aca="false">E6/COUNT('Щоденний облік'!$B$6:$B$35)</f>
         <v>0</v>
       </c>
@@ -2977,9 +5659,17 @@
         <f aca="false">IF(I6=0,"—",INDEX('Щоденний облік'!$B$6:$B$35,MATCH(I6,'Щоденний облік'!$O$6:$O$35,0)))</f>
         <v>—</v>
       </c>
+      <c r="K6" s="8" t="n">
+        <f aca="false">COUNTA('Склад МВГ'!D32:D41)</f>
+        <v>0</v>
+      </c>
+      <c r="L6" s="43" t="n">
+        <f aca="false">'Склад МВГ'!AJ42</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="37" t="s">
+      <c r="A7" s="49" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="16" t="n">
@@ -2998,7 +5688,7 @@
         <f aca="false">'Щоденний облік'!S36</f>
         <v>0</v>
       </c>
-      <c r="F7" s="38" t="n">
+      <c r="F7" s="50" t="n">
         <f aca="false">IF($E$7=0,0,E7/$E$7)</f>
         <v>0</v>
       </c>
@@ -3006,7 +5696,7 @@
         <f aca="false">COUNTIF('Щоденний облік'!$S$6:$S$35,"&gt;0")</f>
         <v>0</v>
       </c>
-      <c r="H7" s="39" t="n">
+      <c r="H7" s="51" t="n">
         <f aca="false">E7/COUNT('Щоденний облік'!$B$6:$B$35)</f>
         <v>0</v>
       </c>
@@ -3014,35 +5704,43 @@
         <f aca="false">MAX('Щоденний облік'!$S$6:$S$35)</f>
         <v>0</v>
       </c>
-      <c r="J7" s="40" t="str">
+      <c r="J7" s="52" t="str">
         <f aca="false">IF(I7=0,"—",INDEX('Щоденний облік'!$B$6:$B$35,MATCH(I7,'Щоденний облік'!$S$6:$S$35,0)))</f>
         <v>—</v>
       </c>
+      <c r="K7" s="17" t="n">
+        <f aca="false">SUM(K4:K6)</f>
+        <v>0</v>
+      </c>
+      <c r="L7" s="17" t="n">
+        <f aca="false">SUM(L4:L6)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="41" t="s">
-        <v>31</v>
+      <c r="A9" s="53" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="30" t="s">
+      <c r="A11" s="42" t="s">
         <v>5</v>
       </c>
       <c r="B11" s="8" t="n">
@@ -3063,7 +5761,7 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="35" t="s">
+      <c r="A12" s="47" t="s">
         <v>6</v>
       </c>
       <c r="B12" s="8" t="n">
@@ -3084,7 +5782,7 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="36" t="s">
+      <c r="A13" s="48" t="s">
         <v>7</v>
       </c>
       <c r="B13" s="8" t="n">
@@ -3105,7 +5803,7 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="37" t="s">
+      <c r="A14" s="49" t="s">
         <v>8</v>
       </c>
       <c r="B14" s="17" t="n">
@@ -3126,13 +5824,13 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="42" t="s">
-        <v>35</v>
+      <c r="A16" s="54" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>